<commit_message>
feat(branding-site): website CMS, product-selection wizard and custom orders
Adds CMS-managed page content + SEO (per-locale hero/body, meta title/
description, canonical, hreflang, JSON-LD, noindex) with admin CRUD over a
new pages table; a /choose 5-question wizard recommending the best-fit
deployment via a new ProductRecommender (app / raw-PHP / WP theme / Node
variant); and a /custom-order form for custom development/modifications/
extra features stored in custom_requests with an admin follow-up inbox.
Adds /products/node marketing surface and '1 license, 4 products' CTAs.

Suite: 123 tests / 349 assertions (new PageTest + ProductRecommenderTest,
extended RouterRegistrationTest). Coverage: docs from
docs/prompts/branding-website-cms-selection-and-custom-orders-prompt.md.
</commit_message>
<xml_diff>
--- a/docs/feature-tracking/branding-website-feature-matrix.xlsx
+++ b/docs/feature-tracking/branding-website-feature-matrix.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G88"/>
+  <dimension ref="A1:G97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -746,12 +746,12 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>About page</t>
+          <t>CMS-driven page hero/content</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Company/about content.</t>
+          <t>Per-page hero heading/intro/body from the pages table, locale-aware; template defaults win until edited.</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -766,7 +766,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>GET /about (web.php:33).</t>
+          <t>app/Models/Page.php + views/site/partials/cms_block.php; Page::forPath() per route.</t>
         </is>
       </c>
     </row>
@@ -781,12 +781,12 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Legal pages (refund policy / terms / privacy)</t>
+          <t>Per-page SEO (title/description/canonical/hreflang/JSON-LD)</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Static legal/legalese pages.</t>
+          <t>CMS-managed metadata merged in main.php layout; per-view overrides win, CMS fills gaps.</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -801,7 +801,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>LegalController routes (web.php:34-36).</t>
+          <t>views/layouts/main.php SEO merge; app/Services/Seo.php hreflang + raw JSON-LD support.</t>
         </is>
       </c>
     </row>
@@ -816,12 +816,12 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Contact page + message form</t>
+          <t>Product-selection wizard (/choose)</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Contact form stores messages to DB.</t>
+          <t>5-question quiz recommending app / raw-PHP / WP theme / Node variant with runner-up + all-product cards.</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>GET/POST /contact (web.php:37-38); inbox in admin.</t>
+          <t>GET/POST /choose (web.php:34-35); ChooseController + ProductRecommender.</t>
         </is>
       </c>
     </row>
@@ -851,12 +851,12 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>robots.txt + sitemap.xml</t>
+          <t>Custom order/development request (/custom-order)</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>SEO outputs in public/.</t>
+          <t>Order custom development, modifications or extra features for any product; stored + emailed to sales.</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -871,7 +871,7 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>public/robots.txt + sitemap.xml present.</t>
+          <t>GET/POST /custom-order (web.php:36-37); CustomOrderController; admin follow-up inbox.</t>
         </is>
       </c>
     </row>
@@ -881,17 +881,17 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Blog</t>
+          <t>Public site</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Blog index (listing + pagination)</t>
+          <t>About page</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Public article list.</t>
+          <t>Company/about content.</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -906,7 +906,7 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>GET /blog SitePostController::index (web.php:41).</t>
+          <t>GET /about (web.php:33).</t>
         </is>
       </c>
     </row>
@@ -916,17 +916,17 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Blog</t>
+          <t>Public site</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Blog category pages</t>
+          <t>Legal pages (refund policy / terms / privacy)</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Articles by category.</t>
+          <t>Static legal/legalese pages.</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -941,7 +941,7 @@
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>GET /blog/category/{slug} (web.php:42).</t>
+          <t>LegalController routes (web.php:34-36).</t>
         </is>
       </c>
     </row>
@@ -951,17 +951,17 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Blog</t>
+          <t>Public site</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Blog post detail</t>
+          <t>Contact page + message form</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Article view.</t>
+          <t>Contact form stores messages to DB.</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -976,7 +976,7 @@
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>GET /blog/{slug} (web.php:43).</t>
+          <t>GET/POST /contact (web.php:37-38); inbox in admin.</t>
         </is>
       </c>
     </row>
@@ -986,17 +986,17 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Blog</t>
+          <t>Public site</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Posts admin CRUD</t>
+          <t>robots.txt + sitemap.xml</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Manage posts (create/edit/delete/publish).</t>
+          <t>SEO outputs in public/.</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -1011,7 +1011,7 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>admin /posts* routes (web.php:110-117).</t>
+          <t>public/robots.txt + sitemap.xml present.</t>
         </is>
       </c>
     </row>
@@ -1026,12 +1026,12 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Post categories admin CRUD</t>
+          <t>Blog index (listing + pagination)</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Manage categories.</t>
+          <t>Public article list.</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>admin /post-categories* routes (web.php:119-126).</t>
+          <t>GET /blog SitePostController::index (web.php:41).</t>
         </is>
       </c>
     </row>
@@ -1056,17 +1056,17 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>i18n &amp; locality</t>
+          <t>Blog</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>en/bn string coverage</t>
+          <t>Blog category pages</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Two locale files (lang/en.php, lang/bn.php).</t>
+          <t>Articles by category.</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -1081,7 +1081,7 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>lang/{en,bn}.php; I18nTest (8 tests).</t>
+          <t>GET /blog/category/{slug} (web.php:42).</t>
         </is>
       </c>
     </row>
@@ -1091,17 +1091,17 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>i18n &amp; locality</t>
+          <t>Blog</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Manual locale switch (/language/{locale})</t>
+          <t>Blog post detail</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Explicit language selector, wins over geo for the session.</t>
+          <t>Article view.</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1116,7 +1116,7 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>GET /language/{locale} (web.php:47); manual switch clears geo_locale.</t>
+          <t>GET /blog/{slug} (web.php:43).</t>
         </is>
       </c>
     </row>
@@ -1126,17 +1126,17 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>i18n &amp; locality</t>
+          <t>Blog</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Geo-detected locale (server + client tz backstop)</t>
+          <t>Posts admin CRUD</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Auto locale via geo-IP plus /language/geo?tz= client backstop (runs once).</t>
+          <t>Manage posts (create/edit/delete/publish).</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1151,7 +1151,7 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>GET /language/geo (web.php:46); GeoLocaleTest (15) + I18nGeoTest (8).</t>
+          <t>admin /posts* routes (web.php:110-117).</t>
         </is>
       </c>
     </row>
@@ -1161,17 +1161,17 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>i18n &amp; locality</t>
+          <t>Blog</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>BD-vs-int locale/currency behaviour</t>
+          <t>Post categories admin CRUD</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>BD visitors get BDT + bKash/Rocket/Nagad; others USD + Stripe/PayPal/Paddle.</t>
+          <t>Manage categories.</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -1186,7 +1186,7 @@
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>CheckoutController derives currency: BD→BDT else USD; gateway list geo-driven.</t>
+          <t>admin /post-categories* routes (web.php:119-126).</t>
         </is>
       </c>
     </row>
@@ -1196,17 +1196,17 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Checkout &amp; payments</t>
+          <t>i18n &amp; locality</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Checkout page</t>
+          <t>en/bn string coverage</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Renders cart + plan selection with local currency.</t>
+          <t>Two locale files (lang/en.php, lang/bn.php).</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -1221,7 +1221,7 @@
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>GET /checkout CheckoutController::index (web.php:50).</t>
+          <t>lang/{en,bn}.php; I18nTest (8 tests).</t>
         </is>
       </c>
     </row>
@@ -1231,17 +1231,17 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Checkout &amp; payments</t>
+          <t>i18n &amp; locality</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Checkout processing</t>
+          <t>Manual locale switch (/language/{locale})</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>POST /checkout creates order + routes to chosen gateway.</t>
+          <t>Explicit language selector, wins over geo for the session.</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -1256,7 +1256,7 @@
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>POST /checkout (web.php:51).</t>
+          <t>GET /language/{locale} (web.php:47); manual switch clears geo_locale.</t>
         </is>
       </c>
     </row>
@@ -1266,17 +1266,17 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Checkout &amp; payments</t>
+          <t>i18n &amp; locality</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Payment status page</t>
+          <t>Geo-detected locale (server + client tz backstop)</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Public status lookup by reference.</t>
+          <t>Auto locale via geo-IP plus /language/geo?tz= client backstop (runs once).</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>GET /checkout/status/{reference} (web.php:52).</t>
+          <t>GET /language/geo (web.php:46); GeoLocaleTest (15) + I18nGeoTest (8).</t>
         </is>
       </c>
     </row>
@@ -1301,17 +1301,17 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Checkout &amp; payments</t>
+          <t>i18n &amp; locality</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Manual (offline) gateway driver</t>
+          <t>BD-vs-int locale/currency behaviour</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Manual payment + admin approval.</t>
+          <t>BD visitors get BDT + bKash/Rocket/Nagad; others USD + Stripe/PayPal/Paddle.</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -1326,7 +1326,7 @@
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>app/Gateways/ManualGateway.php; ManualGatewayTest (2); admin approveManual (web.php:104).</t>
+          <t>CheckoutController derives currency: BD→BDT else USD; gateway list geo-driven.</t>
         </is>
       </c>
     </row>
@@ -1341,12 +1341,12 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Stripe gateway driver</t>
+          <t>Checkout page</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Credit-card checkout via Stripe.</t>
+          <t>Renders cart + plan selection with local currency.</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -1354,14 +1354,14 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F24" s="7" t="inlineStr">
-        <is>
-          <t>Not tested</t>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>app/Gateways/StripeGateway.php; live calls need credentials.</t>
+          <t>GET /checkout CheckoutController::index (web.php:50).</t>
         </is>
       </c>
     </row>
@@ -1376,12 +1376,12 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>PayPal gateway driver</t>
+          <t>Checkout processing</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>PayPal checkout.</t>
+          <t>POST /checkout creates order + routes to chosen gateway.</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -1389,14 +1389,14 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>Not tested</t>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>app/Gateways/PaypalGateway.php; live calls need credentials.</t>
+          <t>POST /checkout (web.php:51).</t>
         </is>
       </c>
     </row>
@@ -1411,12 +1411,12 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Paddle gateway driver</t>
+          <t>Payment status page</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Paddle checkout.</t>
+          <t>Public status lookup by reference.</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -1424,14 +1424,14 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F26" s="7" t="inlineStr">
-        <is>
-          <t>Not tested</t>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>app/Gateways/PaddleGateway.php; live calls need credentials.</t>
+          <t>GET /checkout/status/{reference} (web.php:52).</t>
         </is>
       </c>
     </row>
@@ -1446,12 +1446,12 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>bKash gateway driver (BD)</t>
+          <t>Manual (offline) gateway driver</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>bKash 2-step (create-payment + execute-payment).</t>
+          <t>Manual payment + admin approval.</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -1459,14 +1459,14 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F27" s="7" t="inlineStr">
-        <is>
-          <t>Not tested</t>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>app/Gateways/BkashGateway.php; live calls need credentials.</t>
+          <t>app/Gateways/ManualGateway.php; ManualGatewayTest (2); admin approveManual (web.php:104).</t>
         </is>
       </c>
     </row>
@@ -1481,12 +1481,12 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Rocket gateway driver (BD)</t>
+          <t>Stripe gateway driver</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Rocket payment flow.</t>
+          <t>Credit-card checkout via Stripe.</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -1501,7 +1501,7 @@
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>app/Gateways/RocketGateway.php; live calls need credentials.</t>
+          <t>app/Gateways/StripeGateway.php; live calls need credentials.</t>
         </is>
       </c>
     </row>
@@ -1516,12 +1516,12 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Nagad gateway driver (BD)</t>
+          <t>PayPal gateway driver</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Nagad payment flow.</t>
+          <t>PayPal checkout.</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -1536,7 +1536,7 @@
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>app/Gateways/NagadGateway.php; live calls need credentials.</t>
+          <t>app/Gateways/PaypalGateway.php; live calls need credentials.</t>
         </is>
       </c>
     </row>
@@ -1551,12 +1551,12 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Gateway factory (env-driven selection)</t>
+          <t>Paddle gateway driver</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Picks active driver from config/gateways.php + env.</t>
+          <t>Paddle checkout.</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -1564,14 +1564,14 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F30" s="6" t="inlineStr">
-        <is>
-          <t>Yes</t>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>Not tested</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>app/Gateways/GatewayFactory.php; GatewayFactoryTest (11).</t>
+          <t>app/Gateways/PaddleGateway.php; live calls need credentials.</t>
         </is>
       </c>
     </row>
@@ -1586,12 +1586,12 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>USD→BDT rate for BD pricing</t>
+          <t>bKash gateway driver (BD)</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>GATEWAY_BDT_RATE env derives BDT amounts for BD customers.</t>
+          <t>bKash 2-step (create-payment + execute-payment).</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -1599,14 +1599,14 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F31" s="6" t="inlineStr">
-        <is>
-          <t>Yes</t>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>Not tested</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>config/gateways.php:10 (default 110).env-driven.</t>
+          <t>app/Gateways/BkashGateway.php; live calls need credentials.</t>
         </is>
       </c>
     </row>
@@ -1621,12 +1621,12 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Gateway webhooks (public, signature-verified)</t>
+          <t>Rocket gateway driver (BD)</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>POST /webhooks/{gateway}, CSRF-exempt via bootstrap, signature checks.</t>
+          <t>Rocket payment flow.</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -1641,7 +1641,7 @@
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>web.php:173; live verification needs real gateway sandbox.</t>
+          <t>app/Gateways/RocketGateway.php; live calls need credentials.</t>
         </is>
       </c>
     </row>
@@ -1656,12 +1656,12 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Manual payment approval flow (admin)</t>
+          <t>Nagad gateway driver (BD)</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Approve/reject offline payments and update order status.</t>
+          <t>Nagad payment flow.</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -1669,14 +1669,14 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F33" s="6" t="inlineStr">
-        <is>
-          <t>Yes</t>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>Not tested</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>admin POST /payments/{id}/approve (web.php:104).</t>
+          <t>app/Gateways/NagadGateway.php; live calls need credentials.</t>
         </is>
       </c>
     </row>
@@ -1691,12 +1691,12 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Payments CSV export (admin + account)</t>
+          <t>Gateway factory (env-driven selection)</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Export payments to CSV.</t>
+          <t>Picks active driver from config/gateways.php + env.</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -1711,7 +1711,7 @@
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>admin /payments/export (web.php:102); account /payments/export (web.php:65).</t>
+          <t>app/Gateways/GatewayFactory.php; GatewayFactoryTest (11).</t>
         </is>
       </c>
     </row>
@@ -1721,17 +1721,17 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>License API</t>
+          <t>Checkout &amp; payments</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>GET /api/v1/ping</t>
+          <t>USD→BDT rate for BD pricing</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Heartbeat for license servers.</t>
+          <t>GATEWAY_BDT_RATE env derives BDT amounts for BD customers.</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -1746,7 +1746,7 @@
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>routes/api.php:6; ForceJson enforced.</t>
+          <t>config/gateways.php:10 (default 110).env-driven.</t>
         </is>
       </c>
     </row>
@@ -1756,17 +1756,17 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>License API</t>
+          <t>Checkout &amp; payments</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>POST /api/v1/licenses/activate</t>
+          <t>Gateway webhooks (public, signature-verified)</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Activate a license for a product installation.</t>
+          <t>POST /webhooks/{gateway}, CSRF-exempt via bootstrap, signature checks.</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -1774,14 +1774,14 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F36" s="6" t="inlineStr">
-        <is>
-          <t>Yes</t>
+      <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t>Not tested</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>api.php:7; Throttle:10,1.</t>
+          <t>web.php:173; live verification needs real gateway sandbox.</t>
         </is>
       </c>
     </row>
@@ -1791,17 +1791,17 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>License API</t>
+          <t>Checkout &amp; payments</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>POST /api/v1/licenses/validate</t>
+          <t>Manual payment approval flow (admin)</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Validate a deployed license.</t>
+          <t>Approve/reject offline payments and update order status.</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>api.php:8; Throttle:30,1.</t>
+          <t>admin POST /payments/{id}/approve (web.php:104).</t>
         </is>
       </c>
     </row>
@@ -1826,17 +1826,17 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>License API</t>
+          <t>Checkout &amp; payments</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>POST /api/v1/licenses/deactivate</t>
+          <t>Payments CSV export (admin + account)</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Deactivate an installation.</t>
+          <t>Export payments to CSV.</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>api.php:9; Throttle:10,1.</t>
+          <t>admin /payments/export (web.php:102); account /payments/export (web.php:65).</t>
         </is>
       </c>
     </row>
@@ -1866,12 +1866,12 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>GET /api/v1/licenses/status</t>
+          <t>GET /api/v1/ping</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Query license status.</t>
+          <t>Heartbeat for license servers.</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -1886,7 +1886,7 @@
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>api.php:10; Throttle:30,1.</t>
+          <t>routes/api.php:6; ForceJson enforced.</t>
         </is>
       </c>
     </row>
@@ -1901,12 +1901,12 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>X-Product-Secret signature auth</t>
+          <t>POST /api/v1/licenses/activate</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>License-mutation requests must match X-Product-Secret.</t>
+          <t>Activate a license for a product installation.</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -1921,7 +1921,7 @@
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>LicenseApiController.php:29; LicenseApiSecurityTest (3).</t>
+          <t>api.php:7; Throttle:10,1.</t>
         </is>
       </c>
     </row>
@@ -1936,12 +1936,12 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Endpoint rate limiting</t>
+          <t>POST /api/v1/licenses/validate</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Throttle middleware on all license endpoints.</t>
+          <t>Validate a deployed license.</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>Throttle:&lt;n&gt;,&lt;m&gt; per route; ThrottleMiddleware core.</t>
+          <t>api.php:8; Throttle:30,1.</t>
         </is>
       </c>
     </row>
@@ -1971,12 +1971,12 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>JSON-enforced responses</t>
+          <t>POST /api/v1/licenses/deactivate</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>ForceJsonMiddleware on /api/v1 (no HTML leakage).</t>
+          <t>Deactivate an installation.</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -1991,7 +1991,7 @@
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>api.php group middleware (ForceJsonMiddleware).</t>
+          <t>api.php:9; Throttle:10,1.</t>
         </is>
       </c>
     </row>
@@ -2006,12 +2006,12 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Activity log on license operations</t>
+          <t>GET /api/v1/licenses/status</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Mutations recorded for admin audit view.</t>
+          <t>Query license status.</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>LicenseManager + admin /activities screen.</t>
+          <t>api.php:10; Throttle:30,1.</t>
         </is>
       </c>
     </row>
@@ -2036,17 +2036,17 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>Customer portal</t>
+          <t>License API</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Account dashboard (overview + notifications)</t>
+          <t>X-Product-Secret signature auth</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Authenticated overview with unread notifications.</t>
+          <t>License-mutation requests must match X-Product-Secret.</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>AccountDashboard (web.php:63); mark-read route web.php:78.</t>
+          <t>LicenseApiController.php:29; LicenseApiSecurityTest (3).</t>
         </is>
       </c>
     </row>
@@ -2071,17 +2071,17 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Customer portal</t>
+          <t>License API</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>API token view/regenerate</t>
+          <t>Endpoint rate limiting</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Regenerate the account API token.</t>
+          <t>Throttle middleware on all license endpoints.</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t>POST /api-token/regenerate (web.php:64).</t>
+          <t>Throttle:&lt;n&gt;,&lt;m&gt; per route; ThrottleMiddleware core.</t>
         </is>
       </c>
     </row>
@@ -2106,17 +2106,17 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>Customer portal</t>
+          <t>License API</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Payments list + CSV export</t>
+          <t>JSON-enforced responses</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Own payments + export.</t>
+          <t>ForceJsonMiddleware on /api/v1 (no HTML leakage).</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -2131,7 +2131,7 @@
       </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
-          <t>account /payments (web.php:70) + export (web.php:65).</t>
+          <t>api.php group middleware (ForceJsonMiddleware).</t>
         </is>
       </c>
     </row>
@@ -2141,17 +2141,17 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Customer portal</t>
+          <t>License API</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Licenses list + detail</t>
+          <t>Activity log on license operations</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Owned licenses overview and per-license page.</t>
+          <t>Mutations recorded for admin audit view.</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -2166,7 +2166,7 @@
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>AccountLicense (web.php:66-67).</t>
+          <t>LicenseManager + admin /activities screen.</t>
         </is>
       </c>
     </row>
@@ -2181,12 +2181,12 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>License renewal request</t>
+          <t>Account dashboard (overview + notifications)</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Request license renewal.</t>
+          <t>Authenticated overview with unread notifications.</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -2201,7 +2201,7 @@
       </c>
       <c r="G48" s="4" t="inlineStr">
         <is>
-          <t>POST /licenses/{id}/renew (web.php:68).</t>
+          <t>AccountDashboard (web.php:63); mark-read route web.php:78.</t>
         </is>
       </c>
     </row>
@@ -2216,12 +2216,12 @@
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Activation revoke</t>
+          <t>API token view/regenerate</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>Revoke a device activation.</t>
+          <t>Regenerate the account API token.</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -2236,7 +2236,7 @@
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>POST /activations/revoke (web.php:70).</t>
+          <t>POST /api-token/regenerate (web.php:64).</t>
         </is>
       </c>
     </row>
@@ -2251,12 +2251,12 @@
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Downloads (packages + client documents)</t>
+          <t>Payments list + CSV export</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>Download purchased packages/docs.</t>
+          <t>Own payments + export.</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
-          <t>DownloadController (web.php:75-77).</t>
+          <t>account /payments (web.php:70) + export (web.php:65).</t>
         </is>
       </c>
     </row>
@@ -2286,12 +2286,12 @@
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Settings (profile + preferences)</t>
+          <t>Licenses list + detail</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>Update account settings.</t>
+          <t>Owned licenses overview and per-license page.</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -2306,7 +2306,7 @@
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
-          <t>Settings routes (web.php:71-73).</t>
+          <t>AccountLicense (web.php:66-67).</t>
         </is>
       </c>
     </row>
@@ -2316,17 +2316,17 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Admin backend</t>
+          <t>Customer portal</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Admin dashboard</t>
+          <t>License renewal request</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>Admin overview.</t>
+          <t>Request license renewal.</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -2341,7 +2341,7 @@
       </c>
       <c r="G52" s="4" t="inlineStr">
         <is>
-          <t>AdminDashboard (web.php:83-84).</t>
+          <t>POST /licenses/{id}/renew (web.php:68).</t>
         </is>
       </c>
     </row>
@@ -2351,17 +2351,17 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Admin backend</t>
+          <t>Customer portal</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Customers management</t>
+          <t>Activation revoke</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>List + edit customers.</t>
+          <t>Revoke a device activation.</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -2376,7 +2376,7 @@
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
-          <t>CustomerController (web.php:86-88).</t>
+          <t>POST /activations/revoke (web.php:70).</t>
         </is>
       </c>
     </row>
@@ -2386,17 +2386,17 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>Admin backend</t>
+          <t>Customer portal</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Plans CRUD</t>
+          <t>Downloads (packages + client documents)</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>Create/edit/license plans.</t>
+          <t>Download purchased packages/docs.</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -2411,7 +2411,7 @@
       </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
-          <t>PlanController (web.php:90-94); PlanTest (2).</t>
+          <t>DownloadController (web.php:75-77).</t>
         </is>
       </c>
     </row>
@@ -2421,17 +2421,17 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Admin backend</t>
+          <t>Customer portal</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Licenses management (status + extend)</t>
+          <t>Settings (profile + preferences)</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>Create/license list, update status, extend.</t>
+          <t>Update account settings.</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -2446,7 +2446,7 @@
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
-          <t>AdminLicense (web.php:96-100).</t>
+          <t>Settings routes (web.php:71-73).</t>
         </is>
       </c>
     </row>
@@ -2461,12 +2461,12 @@
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Payments admin + approve + export</t>
+          <t>Admin dashboard</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>List, approve manual, export CSV.</t>
+          <t>Admin overview.</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
-          <t>AdminPayment (web.php:102-104).</t>
+          <t>AdminDashboard (web.php:83-84).</t>
         </is>
       </c>
     </row>
@@ -2496,12 +2496,12 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>Subscriptions overview</t>
+          <t>Customers management</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>Recurring subscriptions list.</t>
+          <t>List + edit customers.</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -2516,7 +2516,7 @@
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
-          <t>SubscriptionController (web.php:105).</t>
+          <t>CustomerController (web.php:86-88).</t>
         </is>
       </c>
     </row>
@@ -2531,12 +2531,12 @@
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>Messages inbox</t>
+          <t>Plans CRUD</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>Contact-form messages + mark read.</t>
+          <t>Create/edit/license plans.</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -2551,7 +2551,7 @@
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
-          <t>MessageController (web.php:128-129).</t>
+          <t>PlanController (web.php:90-94); PlanTest (2).</t>
         </is>
       </c>
     </row>
@@ -2566,12 +2566,12 @@
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Activity log screen</t>
+          <t>Licenses management (status + extend)</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>Audit trail of admin/customer actions.</t>
+          <t>Create/license list, update status, extend.</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -2586,7 +2586,7 @@
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
-          <t>ActivityController (web.php:131).</t>
+          <t>AdminLicense (web.php:96-100).</t>
         </is>
       </c>
     </row>
@@ -2601,12 +2601,12 @@
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Visitor log screen</t>
+          <t>Payments admin + approve + export</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>Visitor paths/locations.</t>
+          <t>List, approve manual, export CSV.</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -2621,7 +2621,7 @@
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
-          <t>VisitorController (web.php:133); VisitorLogTest (8).</t>
+          <t>AdminPayment (web.php:102-104).</t>
         </is>
       </c>
     </row>
@@ -2636,12 +2636,12 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Settings screen</t>
+          <t>Subscriptions overview</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>Site settings + support-widget toggle + contact details.</t>
+          <t>Recurring subscriptions list.</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -2656,7 +2656,7 @@
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
-          <t>SettingsController (web.php:135-136); Settings model defaults.</t>
+          <t>SubscriptionController (web.php:105).</t>
         </is>
       </c>
     </row>
@@ -2671,12 +2671,12 @@
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>Account (profile + password)</t>
+          <t>Messages inbox</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>Admin profile maintenance.</t>
+          <t>Contact-form messages + mark read.</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -2691,7 +2691,7 @@
       </c>
       <c r="G62" s="4" t="inlineStr">
         <is>
-          <t>AccountController (web.php:138-140).</t>
+          <t>MessageController (web.php:128-129).</t>
         </is>
       </c>
     </row>
@@ -2706,12 +2706,12 @@
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>Services config (per-product features)</t>
+          <t>Activity log screen</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>Enable/disable features per product for marketing display.</t>
+          <t>Audit trail of admin/customer actions.</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -2726,7 +2726,7 @@
       </c>
       <c r="G63" s="4" t="inlineStr">
         <is>
-          <t>ServiceController (web.php:142-143).</t>
+          <t>ActivityController (web.php:131).</t>
         </is>
       </c>
     </row>
@@ -2741,12 +2741,12 @@
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>Packages management (send/download/toggle)</t>
+          <t>Visitor log screen</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>Release packages, toggle visibility, send + download.</t>
+          <t>Visitor paths/locations.</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -2761,7 +2761,7 @@
       </c>
       <c r="G64" s="4" t="inlineStr">
         <is>
-          <t>PackageController (web.php:145-149).</t>
+          <t>VisitorController (web.php:133); VisitorLogTest (8).</t>
         </is>
       </c>
     </row>
@@ -2776,12 +2776,12 @@
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>Client documents (send/download)</t>
+          <t>Settings screen</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>Deliver docs to customers.</t>
+          <t>Site settings + support-widget toggle + contact details.</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -2796,7 +2796,7 @@
       </c>
       <c r="G65" s="4" t="inlineStr">
         <is>
-          <t>ClientDocumentController (web.php:151-154).</t>
+          <t>SettingsController (web.php:135-136); Settings model defaults.</t>
         </is>
       </c>
     </row>
@@ -2811,12 +2811,12 @@
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>Email templates editor</t>
+          <t>Account (profile + password)</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>Edit transactional email templates.</t>
+          <t>Admin profile maintenance.</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -2831,7 +2831,7 @@
       </c>
       <c r="G66" s="4" t="inlineStr">
         <is>
-          <t>EmailTemplateController (web.php:156-157).</t>
+          <t>AccountController (web.php:138-140).</t>
         </is>
       </c>
     </row>
@@ -2846,12 +2846,12 @@
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>Push notifications admin + send</t>
+          <t>Services config (per-product features)</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>Create + send push notifications.</t>
+          <t>Enable/disable features per product for marketing display.</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -2866,7 +2866,7 @@
       </c>
       <c r="G67" s="4" t="inlineStr">
         <is>
-          <t>PushNotificationController (web.php:159-161).</t>
+          <t>ServiceController (web.php:142-143).</t>
         </is>
       </c>
     </row>
@@ -2881,12 +2881,12 @@
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>Gateway config screen</t>
+          <t>Packages management (send/download/toggle)</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>Toggle/configure payment gateways.</t>
+          <t>Release packages, toggle visibility, send + download.</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -2901,7 +2901,7 @@
       </c>
       <c r="G68" s="4" t="inlineStr">
         <is>
-          <t>GatewayController (web.php:163-164).</t>
+          <t>PackageController (web.php:145-149).</t>
         </is>
       </c>
     </row>
@@ -2916,12 +2916,12 @@
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>Cache management/clear</t>
+          <t>Client documents (send/download)</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>Cache admin + clear action.</t>
+          <t>Deliver docs to customers.</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -2936,7 +2936,7 @@
       </c>
       <c r="G69" s="4" t="inlineStr">
         <is>
-          <t>CacheController (web.php:166-167).</t>
+          <t>ClientDocumentController (web.php:151-154).</t>
         </is>
       </c>
     </row>
@@ -2951,12 +2951,12 @@
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>Backup (create/download/delete)</t>
+          <t>Email templates editor</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>DB backup management.</t>
+          <t>Edit transactional email templates.</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -2971,7 +2971,7 @@
       </c>
       <c r="G70" s="4" t="inlineStr">
         <is>
-          <t>BackupController (web.php:169-171).</t>
+          <t>EmailTemplateController (web.php:156-157).</t>
         </is>
       </c>
     </row>
@@ -2981,17 +2981,17 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>Support widget</t>
+          <t>Admin backend</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>Support widget on public site</t>
+          <t>Push notifications admin + send</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>Widget partial in main layout.</t>
+          <t>Create + send push notifications.</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -3006,7 +3006,7 @@
       </c>
       <c r="G71" s="4" t="inlineStr">
         <is>
-          <t>views/layouts/main.php:246 support_widget partial; enabled by default.</t>
+          <t>PushNotificationController (web.php:159-161).</t>
         </is>
       </c>
     </row>
@@ -3016,17 +3016,17 @@
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>Support widget</t>
+          <t>Admin backend</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>Widget toggle via settings</t>
+          <t>Gateway config screen</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>Enable/disable from admin settings.</t>
+          <t>Toggle/configure payment gateways.</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -3041,7 +3041,7 @@
       </c>
       <c r="G72" s="4" t="inlineStr">
         <is>
-          <t>Settings key support.widget_enabled (default 1); settings.php:110.</t>
+          <t>GatewayController (web.php:163-164).</t>
         </is>
       </c>
     </row>
@@ -3051,17 +3051,17 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>PWA</t>
+          <t>Admin backend</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>manifest.json</t>
+          <t>Cache management/clear</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>Web-app manifest (public/manifest.json).</t>
+          <t>Cache admin + clear action.</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -3076,7 +3076,7 @@
       </c>
       <c r="G73" s="4" t="inlineStr">
         <is>
-          <t>public/manifest.json present.</t>
+          <t>CacheController (web.php:166-167).</t>
         </is>
       </c>
     </row>
@@ -3086,17 +3086,17 @@
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>PWA</t>
+          <t>Admin backend</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>Service worker (sw.js + register-sw.js)</t>
+          <t>Backup (create/download/delete)</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>Registration script in layout; sw.js cached in public/.</t>
+          <t>DB backup management.</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -3111,7 +3111,7 @@
       </c>
       <c r="G74" s="4" t="inlineStr">
         <is>
-          <t>main.php:264 register-sw.js; public/sw.js.</t>
+          <t>BackupController (web.php:169-171).</t>
         </is>
       </c>
     </row>
@@ -3121,17 +3121,17 @@
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>PWA</t>
+          <t>Website CMS</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>Offline page (offline.html)</t>
+          <t>Pages library (pages table + seeds)</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>Fallback shell shown when offline.</t>
+          <t>pages table with 16 seed rows covering every static/product route; soft delete.</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -3146,7 +3146,7 @@
       </c>
       <c r="G75" s="4" t="inlineStr">
         <is>
-          <t>public/offline.html present.</t>
+          <t>database/schema.sql pages table + seeds; Page model forPath()/routes().</t>
         </is>
       </c>
     </row>
@@ -3156,17 +3156,17 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>PWA</t>
+          <t>Website CMS</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>App icons</t>
+          <t>Pages admin (CRUD + soft delete)</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>Install icons.</t>
+          <t>List/create/edit/delete pages; route + name + sort + active + noindex + JSON-LD fields.</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -3181,7 +3181,7 @@
       </c>
       <c r="G76" s="4" t="inlineStr">
         <is>
-          <t>public/icons/ + apple-touch-icon.</t>
+          <t>PageController (web.php:128-133); views/admin/pages.php + page_form.php.</t>
         </is>
       </c>
     </row>
@@ -3191,17 +3191,17 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>PWA</t>
+          <t>Website CMS</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>PWA test coverage</t>
+          <t>Per-locale body copy (en/bn)</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>PwaTest mocks SW/manifest wiring.</t>
+          <t>Locale columns per page fall back en→bn; locale blank means template default wins.</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -3216,7 +3216,7 @@
       </c>
       <c r="G77" s="4" t="inlineStr">
         <is>
-          <t>tests/Unit/PwaTest.php (6 tests).</t>
+          <t>Page::localized(); page_form locale panels; I18n key parity maintained.</t>
         </is>
       </c>
     </row>
@@ -3226,17 +3226,17 @@
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Website CMS</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>Admin/auth middleware</t>
+          <t>Custom-orders admin inbox + status workflow</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>Admin routes gated; account routes auth-gated.</t>
+          <t>Follow up on custom-order requests: unread badge, mark read, status pipeline, archive.</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -3251,7 +3251,7 @@
       </c>
       <c r="G78" s="4" t="inlineStr">
         <is>
-          <t>AdminMiddleware + AuthMiddleware (app/Core/Middleware).</t>
+          <t>CustomRequestController (web.php:135-139); views/admin/custom_requests.php; CustomRequest::countUnread() badge.</t>
         </is>
       </c>
     </row>
@@ -3261,17 +3261,17 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Support widget</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>Security headers middleware</t>
+          <t>Support widget on public site</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>Outbound security headers.</t>
+          <t>Widget partial in main layout.</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -3286,7 +3286,7 @@
       </c>
       <c r="G79" s="4" t="inlineStr">
         <is>
-          <t>SecurityHeadersMiddleware.</t>
+          <t>views/layouts/main.php:246 support_widget partial; enabled by default.</t>
         </is>
       </c>
     </row>
@@ -3296,17 +3296,17 @@
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Support widget</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>CORS middleware</t>
+          <t>Widget toggle via settings</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>CORS policy for the license API.</t>
+          <t>Enable/disable from admin settings.</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
@@ -3321,7 +3321,7 @@
       </c>
       <c r="G80" s="4" t="inlineStr">
         <is>
-          <t>CorsMiddleware.</t>
+          <t>Settings key support.widget_enabled (default 1); settings.php:110.</t>
         </is>
       </c>
     </row>
@@ -3331,17 +3331,17 @@
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>PWA</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>CSRF protection</t>
+          <t>manifest.json</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>CSRF token issue/validate in bootstrap + core forms.</t>
+          <t>Web-app manifest (public/manifest.json).</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -3356,7 +3356,7 @@
       </c>
       <c r="G81" s="4" t="inlineStr">
         <is>
-          <t>app/Core/bootstrap.php CSRF session handling.</t>
+          <t>public/manifest.json present.</t>
         </is>
       </c>
     </row>
@@ -3366,17 +3366,17 @@
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>PWA</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>Throttle middleware</t>
+          <t>Service worker (sw.js + register-sw.js)</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>Route rate limiting (login, license API, contact).</t>
+          <t>Registration script in layout; sw.js cached in public/.</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
@@ -3391,7 +3391,7 @@
       </c>
       <c r="G82" s="4" t="inlineStr">
         <is>
-          <t>ThrottleMiddleware; applied via route options.</t>
+          <t>main.php:264 register-sw.js; public/sw.js.</t>
         </is>
       </c>
     </row>
@@ -3401,17 +3401,17 @@
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>PWA</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>Locale middleware</t>
+          <t>Offline page (offline.html)</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>Request-locale resolution before controllers.</t>
+          <t>Fallback shell shown when offline.</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -3426,7 +3426,7 @@
       </c>
       <c r="G83" s="4" t="inlineStr">
         <is>
-          <t>LocaleMiddleware.</t>
+          <t>public/offline.html present.</t>
         </is>
       </c>
     </row>
@@ -3436,17 +3436,17 @@
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>PWA</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>XSS hardening in views</t>
+          <t>App icons</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>Escaped output via plain PHP e()/esc helpers.</t>
+          <t>Install icons.</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -3461,7 +3461,7 @@
       </c>
       <c r="G84" s="4" t="inlineStr">
         <is>
-          <t>Views escape dynamic values.</t>
+          <t>public/icons/ + apple-touch-icon.</t>
         </is>
       </c>
     </row>
@@ -3471,17 +3471,17 @@
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>Testing &amp; delivery</t>
+          <t>PWA</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>Unit test suite (103 tests / 12 files)</t>
+          <t>PWA test coverage</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>Core, gateways, models, services, security, PWA, geo, i18n.</t>
+          <t>PwaTest mocks SW/manifest wiring.</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="G85" s="4" t="inlineStr">
         <is>
-          <t>tests/Unit/** — 103 function test across 12 files.</t>
+          <t>tests/Unit/PwaTest.php (6 tests).</t>
         </is>
       </c>
     </row>
@@ -3506,17 +3506,17 @@
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>Testing &amp; delivery</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>Route-registration consistency test</t>
+          <t>Admin/auth middleware</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>RouterRegistrationTest.</t>
+          <t>Admin routes gated; account routes auth-gated.</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
@@ -3531,7 +3531,7 @@
       </c>
       <c r="G86" s="4" t="inlineStr">
         <is>
-          <t>RouterRegistrationTest (15).</t>
+          <t>AdminMiddleware + AuthMiddleware (app/Core/Middleware).</t>
         </is>
       </c>
     </row>
@@ -3541,17 +3541,17 @@
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>Testing &amp; delivery</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>Fake DB for tests</t>
+          <t>Security headers middleware</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>Isolated test backend.</t>
+          <t>Outbound security headers.</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
@@ -3566,7 +3566,7 @@
       </c>
       <c r="G87" s="4" t="inlineStr">
         <is>
-          <t>tests/FakeDatabase.php.</t>
+          <t>SecurityHeadersMiddleware.</t>
         </is>
       </c>
     </row>
@@ -3576,30 +3576,345 @@
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C88" s="4" t="inlineStr">
+        <is>
+          <t>CORS middleware</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>CORS policy for the license API.</t>
+        </is>
+      </c>
+      <c r="E88" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F88" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G88" s="4" t="inlineStr">
+        <is>
+          <t>CorsMiddleware.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C89" s="4" t="inlineStr">
+        <is>
+          <t>CSRF protection</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>CSRF token issue/validate in bootstrap + core forms.</t>
+        </is>
+      </c>
+      <c r="E89" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F89" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G89" s="4" t="inlineStr">
+        <is>
+          <t>app/Core/bootstrap.php CSRF session handling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C90" s="4" t="inlineStr">
+        <is>
+          <t>Throttle middleware</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>Route rate limiting (login, license API, contact).</t>
+        </is>
+      </c>
+      <c r="E90" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F90" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G90" s="4" t="inlineStr">
+        <is>
+          <t>ThrottleMiddleware; applied via route options.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C91" s="4" t="inlineStr">
+        <is>
+          <t>Locale middleware</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>Request-locale resolution before controllers.</t>
+        </is>
+      </c>
+      <c r="E91" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F91" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G91" s="4" t="inlineStr">
+        <is>
+          <t>LocaleMiddleware.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C92" s="4" t="inlineStr">
+        <is>
+          <t>XSS hardening in views</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>Escaped output via plain PHP e()/esc helpers.</t>
+        </is>
+      </c>
+      <c r="E92" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F92" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G92" s="4" t="inlineStr">
+        <is>
+          <t>Views escape dynamic values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
           <t>Testing &amp; delivery</t>
         </is>
       </c>
-      <c r="C88" s="4" t="inlineStr">
+      <c r="C93" s="4" t="inlineStr">
+        <is>
+          <t>Unit test suite (123 tests / 14 files)</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="inlineStr">
+        <is>
+          <t>Core, gateways, models, services, security, PWA, geo, i18n.</t>
+        </is>
+      </c>
+      <c r="E93" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F93" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G93" s="4" t="inlineStr">
+        <is>
+          <t>tests/Unit/** — 123 function test across 14 files.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>Testing &amp; delivery</t>
+        </is>
+      </c>
+      <c r="C94" s="4" t="inlineStr">
+        <is>
+          <t>Route-registration consistency test</t>
+        </is>
+      </c>
+      <c r="D94" s="4" t="inlineStr">
+        <is>
+          <t>RouterRegistrationTest.</t>
+        </is>
+      </c>
+      <c r="E94" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F94" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G94" s="4" t="inlineStr">
+        <is>
+          <t>RouterRegistrationTest (17).</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>Testing &amp; delivery</t>
+        </is>
+      </c>
+      <c r="C95" s="4" t="inlineStr">
+        <is>
+          <t>CMS/quiz/custom-order model+service tests</t>
+        </is>
+      </c>
+      <c r="D95" s="4" t="inlineStr">
+        <is>
+          <t>PageTest + ProductRecommenderTest.</t>
+        </is>
+      </c>
+      <c r="E95" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F95" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G95" s="4" t="inlineStr">
+        <is>
+          <t>PageTest (9) + ProductRecommenderTest (9).</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>Testing &amp; delivery</t>
+        </is>
+      </c>
+      <c r="C96" s="4" t="inlineStr">
+        <is>
+          <t>Fake DB for tests</t>
+        </is>
+      </c>
+      <c r="D96" s="4" t="inlineStr">
+        <is>
+          <t>Isolated test backend.</t>
+        </is>
+      </c>
+      <c r="E96" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F96" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G96" s="4" t="inlineStr">
+        <is>
+          <t>tests/FakeDatabase.php.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>Testing &amp; delivery</t>
+        </is>
+      </c>
+      <c r="C97" s="4" t="inlineStr">
         <is>
           <t>CI: branding tests + export gate</t>
         </is>
       </c>
-      <c r="D88" s="4" t="inlineStr">
+      <c r="D97" s="4" t="inlineStr">
         <is>
           <t>Workflow runs the branding suite and checks int zip + bn leak.</t>
         </is>
       </c>
-      <c r="E88" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F88" s="6" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G88" s="4" t="inlineStr">
+      <c r="E97" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F97" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G97" s="4" t="inlineStr">
         <is>
           <t>.github/workflows/ci.yml 'eskoofy-branding-website Tests' job + artifact checks.</t>
         </is>
@@ -3667,7 +3982,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="C5" s="10" t="n">
         <v>100</v>
@@ -3706,7 +4021,7 @@
         </is>
       </c>
       <c r="B8" s="9" t="n">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="C8" s="9" t="n">
         <v>100</v>
@@ -3743,10 +4058,10 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="C12" s="10" t="n">
-        <v>92</v>
+        <v>92.7</v>
       </c>
     </row>
     <row r="13">
@@ -3759,7 +4074,7 @@
         <v>7</v>
       </c>
       <c r="C13" s="10" t="n">
-        <v>8</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="14">
@@ -3814,7 +4129,7 @@
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
@@ -3829,7 +4144,7 @@
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
@@ -3844,7 +4159,7 @@
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
@@ -3859,7 +4174,7 @@
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
@@ -3874,7 +4189,7 @@
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
@@ -3889,7 +4204,7 @@
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
@@ -3904,7 +4219,7 @@
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>

</xml_diff>